<commit_message>
Add new executable and zip files, remove obsolete executable, and update HTML template
- Added new executable: Correos Salud Interactiva.exe
- Added new zip file: Correos Salud Interactiva.zip
- Removed obsolete executable: CorreosETS.exe
- Created log file for email sending: log_envio_20260224_135322.txt
- Added multiple image assets for email template
- Introduced new HTML template for "carta MH Grupo Salinas" with dynamic placeholders
- Added additional images for footer and header in the email template
</commit_message>
<xml_diff>
--- a/CorreosPrueba.xlsx
+++ b/CorreosPrueba.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\OneDrive\Documentos\Python\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Roberto Monjardin\Desktop\Salud Interactiva\projects\FarmaLeal-Mailing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47DCD44C-0B33-41FF-91B1-8177EDF95BD9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FEC50E4-A46E-45C6-BCE1-AD8B275CAAD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{4BA2E16D-4279-4C2D-B67B-FABFD3AF7B1D}"/>
+    <workbookView xWindow="24024" yWindow="996" windowWidth="21600" windowHeight="11292" xr2:uid="{4BA2E16D-4279-4C2D-B67B-FABFD3AF7B1D}"/>
   </bookViews>
   <sheets>
     <sheet name="Mailing" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
   <si>
     <t xml:space="preserve">Roberto Edgar Monjardin Alvarado </t>
   </si>
@@ -41,35 +41,17 @@
     <t>robertomonjardin95@gmail.com</t>
   </si>
   <si>
-    <t>Escuela en Tecnologías Sustentables</t>
+    <t>rmonjardin@farmaleal.com.mx</t>
   </si>
   <si>
-    <t>dciluminacion@outlook.com</t>
-  </si>
-  <si>
-    <t>gmzdgadriana@gmail.com</t>
-  </si>
-  <si>
-    <t>Adriana Gómez de Gabriel</t>
-  </si>
-  <si>
-    <t>Manuel Rivera Rodríguez</t>
-  </si>
-  <si>
-    <t>evanpenn6@gmail.com</t>
-  </si>
-  <si>
-    <t>ale130393@live.com</t>
-  </si>
-  <si>
-    <t>Alejandra Torres</t>
+    <t>monjardinspotify@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -89,13 +71,6 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -158,41 +133,40 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -213,9 +187,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -253,7 +227,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -359,7 +333,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -501,7 +475,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -526,172 +500,162 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="11"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>7</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="2"/>
       <c r="H5" s="1"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B6" s="5"/>
+      <c r="B6" s="3"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="5"/>
+      <c r="B7" s="3"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="5"/>
+      <c r="B8" s="3"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="5"/>
+      <c r="B9" s="3"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="5"/>
+      <c r="B10" s="3"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="5"/>
+      <c r="B11" s="3"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B12" s="5"/>
+      <c r="B12" s="3"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B13" s="5"/>
+      <c r="B13" s="3"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B14" s="5"/>
+      <c r="B14" s="3"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B15" s="6"/>
+      <c r="B15" s="4"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B16" s="5"/>
+      <c r="B16" s="3"/>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B17" s="5"/>
+      <c r="B17" s="3"/>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B18" s="5"/>
+      <c r="B18" s="3"/>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B19" s="5"/>
+      <c r="B19" s="3"/>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B20" s="5"/>
+      <c r="B20" s="3"/>
     </row>
     <row r="21" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B21" s="5"/>
+      <c r="B21" s="3"/>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B22" s="5"/>
+      <c r="B22" s="3"/>
     </row>
     <row r="23" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B23" s="7"/>
+      <c r="B23" s="5"/>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B24" s="8"/>
+      <c r="B24" s="6"/>
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B25" s="7"/>
+      <c r="B25" s="5"/>
     </row>
     <row r="26" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B26" s="9"/>
+      <c r="B26" s="7"/>
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B27" s="10"/>
+      <c r="B27" s="8"/>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B28" s="11"/>
+      <c r="B28" s="9"/>
     </row>
     <row r="29" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B29" s="11"/>
+      <c r="B29" s="9"/>
     </row>
     <row r="30" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B30" s="11"/>
+      <c r="B30" s="9"/>
     </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B31" s="9"/>
+      <c r="B31" s="7"/>
     </row>
     <row r="32" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B32" s="9"/>
+      <c r="B32" s="7"/>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B33" s="9"/>
+      <c r="B33" s="7"/>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B34" s="12"/>
+      <c r="B34" s="10"/>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B35" s="12"/>
+      <c r="B35" s="10"/>
     </row>
     <row r="36" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B36" s="12"/>
+      <c r="B36" s="10"/>
     </row>
     <row r="37" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B37" s="5"/>
+      <c r="B37" s="3"/>
     </row>
     <row r="38" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B38" s="5"/>
+      <c r="B38" s="3"/>
     </row>
     <row r="39" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B39" s="5"/>
+      <c r="B39" s="3"/>
     </row>
     <row r="40" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B40" s="5"/>
+      <c r="B40" s="3"/>
     </row>
     <row r="41" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B41" s="5"/>
+      <c r="B41" s="3"/>
     </row>
     <row r="42" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B42" s="5"/>
+      <c r="B42" s="3"/>
     </row>
     <row r="43" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B43" s="7"/>
+      <c r="B43" s="5"/>
     </row>
     <row r="44" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B44" s="5"/>
+      <c r="B44" s="3"/>
     </row>
     <row r="45" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B45" s="5"/>
+      <c r="B45" s="3"/>
     </row>
     <row r="46" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B46" s="6"/>
+      <c r="B46" s="4"/>
     </row>
     <row r="47" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B47" s="5"/>
+      <c r="B47" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B1" r:id="rId1" xr:uid="{1F93DB1E-3D44-44F2-B002-2FD2DCB3AB3B}"/>
-    <hyperlink ref="B2" r:id="rId2" xr:uid="{D2C37A59-EA36-4C7A-B7B3-3FC5929DC7C7}"/>
-    <hyperlink ref="B3" r:id="rId3" xr:uid="{794C6460-C40B-452D-AE50-B1BC7572E863}"/>
-    <hyperlink ref="B4" r:id="rId4" xr:uid="{EBBAAE6A-4835-41C3-B9ED-506F78E1E862}"/>
-    <hyperlink ref="B5" r:id="rId5" xr:uid="{87ACEED2-753E-4B17-9836-D002DBABBD93}"/>
+    <hyperlink ref="B2" r:id="rId2" xr:uid="{99850294-73AC-4A34-80AD-9803BFFE1D60}"/>
+    <hyperlink ref="B3" r:id="rId3" xr:uid="{FAA83957-BE05-46D3-AC4A-0B333352AD78}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId6"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>